<commit_message>
Update data: 19 Juli 2026 pukul 18.47 WITA
</commit_message>
<xml_diff>
--- a/dashboard/public/Report_Dashboard_Evening.xlsx
+++ b/dashboard/public/Report_Dashboard_Evening.xlsx
@@ -610,7 +610,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Pukul        : 18.00 WITA</t>
+          <t>Pukul        : 18.47 WITA</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -1911,7 +1911,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Pukul        : 18.00 WITA</t>
+          <t>Pukul        : 18.47 WITA</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -8160,7 +8160,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Pukul        : 18.00 WITA</t>
+          <t>Pukul        : 18.47 WITA</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -9371,7 +9371,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Pukul        : 18.00 WITA</t>
+          <t>Pukul        : 18.47 WITA</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Update data: 19 Juli 2026 pukul 19.58 WITA
</commit_message>
<xml_diff>
--- a/dashboard/public/Report_Dashboard_Evening.xlsx
+++ b/dashboard/public/Report_Dashboard_Evening.xlsx
@@ -610,7 +610,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Pukul        : 18.47 WITA</t>
+          <t>Pukul        : 19.58 WITA</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -1911,7 +1911,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Pukul        : 18.47 WITA</t>
+          <t>Pukul        : 19.58 WITA</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -4876,7 +4876,7 @@
       </c>
       <c r="D68" s="9" t="inlineStr">
         <is>
-          <t>Suharsi</t>
+          <t>Begin</t>
         </is>
       </c>
       <c r="E68" s="9" t="n">
@@ -6145,7 +6145,7 @@
       </c>
       <c r="D95" s="9" t="inlineStr">
         <is>
-          <t>Suharsi</t>
+          <t>Begin</t>
         </is>
       </c>
       <c r="E95" s="9" t="n">
@@ -6427,7 +6427,7 @@
       </c>
       <c r="D101" s="9" t="inlineStr">
         <is>
-          <t>Suharsi</t>
+          <t>Begin</t>
         </is>
       </c>
       <c r="E101" s="9" t="n">
@@ -7179,7 +7179,7 @@
       </c>
       <c r="D117" s="9" t="inlineStr">
         <is>
-          <t>Suharsi</t>
+          <t>Begin</t>
         </is>
       </c>
       <c r="E117" s="9" t="n">
@@ -7978,7 +7978,7 @@
       </c>
       <c r="D134" s="9" t="inlineStr">
         <is>
-          <t>Suharsi</t>
+          <t>Begin</t>
         </is>
       </c>
       <c r="E134" s="9" t="n">
@@ -8160,7 +8160,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Pukul        : 18.47 WITA</t>
+          <t>Pukul        : 19.58 WITA</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -9292,7 +9292,7 @@
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>Suharsi</t>
+          <t>Begin</t>
         </is>
       </c>
       <c r="E29" s="9" t="n">
@@ -9371,7 +9371,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Pukul        : 18.47 WITA</t>
+          <t>Pukul        : 19.58 WITA</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">

</xml_diff>